<commit_message>
add: Validacion valores en pedidos y cotizaciones, reducion de los tiempos de carga del excel de terceros y dinarap, y crud de la nueva entidad ad_info_adicional.
</commit_message>
<xml_diff>
--- a/api/src/main/resources/importaciones/CargarFacturas.xlsx
+++ b/api/src/main/resources/importaciones/CargarFacturas.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ismael\Documents\calero-app-desktop\api\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ismael\Documents\calero-app-desktop\api\src\main\resources\importaciones\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7801A396-D69D-44D0-B851-CC711444FDA4}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE2E2FFB-0CFD-45F9-96FE-0B0D07EE7943}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" xr2:uid="{D556B04B-A296-4224-AEE4-E6FD1C8884D2}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="84">
   <si>
     <t>Serie</t>
   </si>
@@ -270,14 +270,20 @@
     <t>Codigo Porcentaje</t>
   </si>
   <si>
-    <t>01/06/2026</t>
+    <t>10/06/2026</t>
+  </si>
+  <si>
+    <t>Forma Pago Sri</t>
+  </si>
+  <si>
+    <t>01</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -317,14 +323,6 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -347,7 +345,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -366,7 +364,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
@@ -684,25 +681,28 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5FC5188F-10D9-41D2-A6FE-2A6D06081501}">
-  <dimension ref="A1:AP16"/>
+  <dimension ref="A1:AQ16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="35.140625" style="20" customWidth="1"/>
+    <col min="3" max="3" width="35.140625" style="19" customWidth="1"/>
     <col min="5" max="5" width="17.28515625" customWidth="1"/>
     <col min="6" max="6" width="22.85546875" customWidth="1"/>
     <col min="7" max="7" width="16.28515625" customWidth="1"/>
     <col min="21" max="21" width="15.28515625" customWidth="1"/>
     <col min="22" max="22" width="28" customWidth="1"/>
+    <col min="24" max="24" width="20.7109375" customWidth="1"/>
+    <col min="28" max="28" width="26" customWidth="1"/>
+    <col min="43" max="43" width="15.85546875" style="19" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="19" t="s">
+      <c r="C1" s="18" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
@@ -822,8 +822,11 @@
       <c r="AP1" s="1" t="s">
         <v>33</v>
       </c>
+      <c r="AQ1" s="18" t="s">
+        <v>82</v>
+      </c>
     </row>
-    <row r="2" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>34</v>
       </c>
@@ -894,7 +897,9 @@
       <c r="Z2" s="7">
         <v>45383</v>
       </c>
-      <c r="AA2" s="9"/>
+      <c r="AA2" s="9">
+        <v>10</v>
+      </c>
       <c r="AB2" s="10" t="s">
         <v>45</v>
       </c>
@@ -912,8 +917,11 @@
       <c r="AN2" s="9"/>
       <c r="AO2" s="9"/>
       <c r="AP2" s="9"/>
+      <c r="AQ2" s="19" t="s">
+        <v>83</v>
+      </c>
     </row>
-    <row r="3" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>34</v>
       </c>
@@ -984,7 +992,9 @@
       <c r="Z3" s="7">
         <v>45383</v>
       </c>
-      <c r="AA3" s="9"/>
+      <c r="AA3" s="9">
+        <v>0</v>
+      </c>
       <c r="AB3" s="9"/>
       <c r="AC3" s="9"/>
       <c r="AD3" s="9"/>
@@ -1000,8 +1010,11 @@
       <c r="AN3" s="9"/>
       <c r="AO3" s="9"/>
       <c r="AP3" s="9"/>
+      <c r="AQ3" s="19" t="s">
+        <v>83</v>
+      </c>
     </row>
-    <row r="4" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>34</v>
       </c>
@@ -1072,7 +1085,9 @@
       <c r="Z4" s="7">
         <v>45383</v>
       </c>
-      <c r="AA4" s="9"/>
+      <c r="AA4" s="9">
+        <v>15</v>
+      </c>
       <c r="AB4" s="9"/>
       <c r="AC4" s="9"/>
       <c r="AD4" s="9"/>
@@ -1088,8 +1103,11 @@
       <c r="AN4" s="9"/>
       <c r="AO4" s="9"/>
       <c r="AP4" s="9"/>
+      <c r="AQ4" s="19" t="s">
+        <v>83</v>
+      </c>
     </row>
-    <row r="5" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>34</v>
       </c>
@@ -1158,7 +1176,9 @@
       <c r="Z5" s="7">
         <v>45383</v>
       </c>
-      <c r="AA5" s="9"/>
+      <c r="AA5" s="9">
+        <v>45</v>
+      </c>
       <c r="AB5" s="9"/>
       <c r="AC5" s="9"/>
       <c r="AD5" s="9"/>
@@ -1174,8 +1194,11 @@
       <c r="AN5" s="9"/>
       <c r="AO5" s="9"/>
       <c r="AP5" s="9"/>
+      <c r="AQ5" s="19" t="s">
+        <v>83</v>
+      </c>
     </row>
-    <row r="6" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>34</v>
       </c>
@@ -1246,7 +1269,9 @@
       <c r="Z6" s="7">
         <v>45383</v>
       </c>
-      <c r="AA6" s="9"/>
+      <c r="AA6" s="9">
+        <v>30</v>
+      </c>
       <c r="AB6" s="9"/>
       <c r="AC6" s="9"/>
       <c r="AD6" s="9"/>
@@ -1262,8 +1287,11 @@
       <c r="AN6" s="9"/>
       <c r="AO6" s="9"/>
       <c r="AP6" s="9"/>
+      <c r="AQ6" s="19" t="s">
+        <v>83</v>
+      </c>
     </row>
-    <row r="7" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>34</v>
       </c>
@@ -1334,7 +1362,9 @@
       <c r="Z7" s="7">
         <v>45383</v>
       </c>
-      <c r="AA7" s="9"/>
+      <c r="AA7" s="9">
+        <v>15</v>
+      </c>
       <c r="AB7" s="9"/>
       <c r="AC7" s="9"/>
       <c r="AD7" s="9"/>
@@ -1350,8 +1380,11 @@
       <c r="AN7" s="9"/>
       <c r="AO7" s="9"/>
       <c r="AP7" s="9"/>
+      <c r="AQ7" s="19" t="s">
+        <v>83</v>
+      </c>
     </row>
-    <row r="8" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
         <v>34</v>
       </c>
@@ -1436,8 +1469,11 @@
       <c r="AN8" s="9"/>
       <c r="AO8" s="9"/>
       <c r="AP8" s="9"/>
+      <c r="AQ8" s="19" t="s">
+        <v>83</v>
+      </c>
     </row>
-    <row r="9" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>34</v>
       </c>
@@ -1522,8 +1558,11 @@
       <c r="AN9" s="9"/>
       <c r="AO9" s="9"/>
       <c r="AP9" s="9"/>
+      <c r="AQ9" s="19" t="s">
+        <v>83</v>
+      </c>
     </row>
-    <row r="10" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>34</v>
       </c>
@@ -1604,8 +1643,11 @@
       <c r="AN10" s="9"/>
       <c r="AO10" s="9"/>
       <c r="AP10" s="9"/>
+      <c r="AQ10" s="19" t="s">
+        <v>83</v>
+      </c>
     </row>
-    <row r="11" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A11" s="9"/>
       <c r="B11" s="9"/>
       <c r="C11" s="17"/>
@@ -1649,10 +1691,10 @@
       <c r="AO11" s="9"/>
       <c r="AP11" s="9"/>
     </row>
-    <row r="12" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A12" s="9"/>
       <c r="B12" s="9"/>
-      <c r="C12" s="17"/>
+      <c r="C12" s="9"/>
       <c r="D12" s="9"/>
       <c r="E12" s="9"/>
       <c r="F12" s="9"/>
@@ -1692,14 +1734,15 @@
       <c r="AN12" s="9"/>
       <c r="AO12" s="9"/>
       <c r="AP12" s="9"/>
+      <c r="AQ12" s="9"/>
     </row>
-    <row r="13" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A13" s="9"/>
       <c r="B13" s="9"/>
-      <c r="C13" s="17"/>
+      <c r="C13" s="9"/>
       <c r="D13" s="9"/>
-      <c r="E13" s="18"/>
-      <c r="F13" s="17"/>
+      <c r="E13" s="9"/>
+      <c r="F13" s="9"/>
       <c r="G13" s="9"/>
       <c r="H13" s="9"/>
       <c r="I13" s="9"/>
@@ -1713,13 +1756,13 @@
       <c r="Q13" s="9"/>
       <c r="R13" s="9"/>
       <c r="S13" s="9"/>
-      <c r="T13" s="10"/>
-      <c r="U13" s="10"/>
-      <c r="V13" s="10"/>
+      <c r="T13" s="9"/>
+      <c r="U13" s="9"/>
+      <c r="V13" s="9"/>
       <c r="W13" s="9"/>
       <c r="X13" s="9"/>
       <c r="Y13" s="9"/>
-      <c r="Z13" s="7"/>
+      <c r="Z13" s="9"/>
       <c r="AA13" s="9"/>
       <c r="AB13" s="9"/>
       <c r="AC13" s="9"/>
@@ -1736,8 +1779,9 @@
       <c r="AN13" s="9"/>
       <c r="AO13" s="9"/>
       <c r="AP13" s="9"/>
+      <c r="AQ13" s="9"/>
     </row>
-    <row r="14" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A14" s="9"/>
       <c r="B14" s="9"/>
       <c r="C14" s="17"/>
@@ -1781,7 +1825,7 @@
       <c r="AO14" s="9"/>
       <c r="AP14" s="9"/>
     </row>
-    <row r="15" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A15" s="9"/>
       <c r="B15" s="9"/>
       <c r="C15" s="17"/>
@@ -1825,7 +1869,7 @@
       <c r="AO15" s="9"/>
       <c r="AP15" s="9"/>
     </row>
-    <row r="16" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A16" s="9"/>
       <c r="B16" s="9"/>
       <c r="C16" s="17"/>

</xml_diff>